<commit_message>
VRPA-00000: Update keywords logic to use wildcards and update excel file as well
</commit_message>
<xml_diff>
--- a/data/Variables-used-by-LLMs.xlsx
+++ b/data/Variables-used-by-LLMs.xlsx
@@ -1,15 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="21029"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC12E10-BCB1-46B1-92A2-AC1B4F8B3797}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8868" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8868" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LLM-selection" sheetId="1" r:id="rId1"/>
-    <sheet name="Common-keywords" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="LLM-selection" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Keyword-mapping" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -36,65 +35,65 @@
     <t>Resume review</t>
   </si>
   <si>
-    <t>forklift</t>
-  </si>
-  <si>
-    <t>fork-lift</t>
-  </si>
-  <si>
-    <t>fork lift</t>
-  </si>
-  <si>
-    <t>labourer</t>
-  </si>
-  <si>
-    <t>packer</t>
-  </si>
-  <si>
-    <t>meat</t>
-  </si>
-  <si>
-    <t>pick</t>
-  </si>
-  <si>
-    <t>pack</t>
-  </si>
-  <si>
-    <t>pick packer</t>
-  </si>
-  <si>
-    <t>picker</t>
-  </si>
-  <si>
-    <t>LO Operator</t>
-  </si>
-  <si>
-    <t>LO</t>
-  </si>
-  <si>
-    <t>civil labourer</t>
-  </si>
-  <si>
-    <t>production worker</t>
-  </si>
-  <si>
-    <t>production</t>
-  </si>
-  <si>
-    <t>worker</t>
+    <t>Role Type</t>
+  </si>
+  <si>
+    <t>Keywords</t>
+  </si>
+  <si>
+    <t>Pick/Packer</t>
+  </si>
+  <si>
+    <t>pack* OR pick*</t>
+  </si>
+  <si>
+    <t>Forklift</t>
+  </si>
+  <si>
+    <t>fork*</t>
+  </si>
+  <si>
+    <t>Labourer/Production</t>
+  </si>
+  <si>
+    <t>production* OR labour*</t>
+  </si>
+  <si>
+    <t>Civil Labourer</t>
+  </si>
+  <si>
+    <t>"civil labourer"</t>
+  </si>
+  <si>
+    <t>Meat Labourer</t>
+  </si>
+  <si>
+    <t>meat OR pack* OR labour* OR production</t>
+  </si>
+  <si>
+    <t>Assembler</t>
+  </si>
+  <si>
+    <t>production OR labour* OR hand tools</t>
+  </si>
+  <si>
+    <t>Bulk Picker</t>
+  </si>
+  <si>
+    <t>pack* OR pick* OR labour* OR bulk</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -457,14 +456,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="57" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -472,7 +471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -480,7 +479,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -488,7 +487,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -498,97 +497,81 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="B8" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>